<commit_message>
Considerando IVU y Moral como catedra
</commit_message>
<xml_diff>
--- a/datos/Malla_Curricular_LLYA.xlsx
+++ b/datos/Malla_Curricular_LLYA.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="25028"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="20417"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Consumo_horas_educacion_secundaria\datos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{024B4E04-5757-437C-BE6D-35C849F1C0B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C98CB854-F388-40C5-9E72-010A40BBEC95}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,15 +20,6 @@
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
     <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
       <xlwcv:version setVersion="1"/>
     </ext>
@@ -37,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="586" uniqueCount="91">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="585" uniqueCount="91">
   <si>
     <t>PROGRAMA</t>
   </si>
@@ -781,18 +772,16 @@
         <v>20</v>
       </c>
       <c r="J4" s="5">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K4" s="5">
         <v>2</v>
       </c>
       <c r="L4" s="4">
         <f t="shared" si="0"/>
-        <v>4</v>
-      </c>
-      <c r="M4" s="5" t="s">
-        <v>21</v>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="M4" s="5"/>
       <c r="N4" s="5" t="s">
         <v>21</v>
       </c>

</xml_diff>

<commit_message>
Actualización de planes de estudio
</commit_message>
<xml_diff>
--- a/datos/Malla_Curricular_LLYA.xlsx
+++ b/datos/Malla_Curricular_LLYA.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Consumo_horas_educacion_secundaria\datos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{262D75B8-1845-48EA-99AD-D1B3DCE8DEDC}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1FE49ACF-1D0A-458B-A11E-DEEB9370E010}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3320,7 +3320,7 @@
         <v>28</v>
       </c>
       <c r="I58" s="5" t="s">
-        <v>33</v>
+        <v>20</v>
       </c>
       <c r="J58" s="5">
         <v>2</v>
@@ -3333,10 +3333,10 @@
         <v>4</v>
       </c>
       <c r="M58" s="5" t="s">
-        <v>33</v>
+        <v>21</v>
       </c>
       <c r="N58" s="5" t="s">
-        <v>33</v>
+        <v>21</v>
       </c>
       <c r="O58" s="5" t="s">
         <v>22</v>
@@ -15865,6 +15865,7 @@
       <c r="O1000" s="4"/>
     </row>
   </sheetData>
+  <autoFilter ref="A1:O66" xr:uid="{437749D5-0DDE-4276-9DD6-17B2BC08D6F2}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>